<commit_message>
qPCR panel: primers for the eight growth-machinery, glucose and response targets (pan-actin design)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/qpcr-additional/qPCR_validation_panel_HS6_vs_4.xlsx
+++ b/downloads/qpcr-additional/qPCR_validation_panel_HS6_vs_4.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Selection logic" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 New primers (5 genes)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 New primers (13 genes)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Full panel" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Design checks" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -39,7 +39,7 @@
       <name val="Consolas"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
         <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -110,12 +105,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -731,7 +720,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Proposed (primers not yet designed)</t>
+          <t>Primers designed (this update)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -801,7 +790,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Proposed (primers not yet designed)</t>
+          <t>Primers designed (this update)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -836,7 +825,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>1 existing + 2 proposed</t>
+          <t>1 existing + 2 new</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -908,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1463,6 +1452,686 @@
       <c r="U6" s="2" t="inlineStr">
         <is>
           <t>AGTCGGCGACCCTTTCTTTCGCGAGCGTTGGCTTAGCAAGGATCGACAAGAGACAAAGCTCGAACGAACGATCGGCGAGGGAGGGCGCTCTTGAAGTGCATTT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>g1305</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>g1305.t1</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Actin; M3 growth machinery (strongest GO signal)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>7.50108995036688e-20</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>-1.92</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>pan-actin: conserved in all 4 copies (g1305, g13337, g13659, g1757); measures total actin</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>family-specific: 100% match at exactly the 4 actin loci, no other site; NOT g1305-specific</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>CCCATCTACGAGGGTTACGC</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>GTGGTGGTGAAGGAGTAGCC</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>119</v>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>4 / 4</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="R7" s="8" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="S7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="8" t="inlineStr">
+        <is>
+          <t>CCCATCTACGAGGGTTACGCTCTCCCGCACGCCGTTCTCCGTATCGATCTTGCCGGCCGTGACCTCACCGACTACATGATGAAGATCCTCACCGAGCGTGGCTACTCCTTCACCACCAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>g8048</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>g8048.t1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Myosin-6; M3 growth machinery</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1.61906919291573e-10</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>GTGCTTCAAGTTGTGGCAGG</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>AGGGCTCTTTCCAGTGCATC</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>164</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>GTGCTTCAAGTTGTGGCAGGCGTGCTCCACCTTGGTAATATCCGATTCTCTGGAGGTGCACGTGGAGAGGGTGCACGTGTTGCTTCTAAAGGCTCCTCAATGTTGGCGTGTGCTGCATGTTGTGATCTACTGGAGCTTGATGCTGATGCACTGGAAAGAGCCCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>g8072</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>g8072.t1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Myosin-I heavy chain; M3 growth machinery</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1.08697695779639e-07</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>CTCAGCAAATCTTCGCGAGC</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>TGTCTTTGCGTTGCCGAAAG</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>CTCAGCAAATCTTCGCGAGCAGATCTTGGAGGCCAACCCTCTCATGGAGGCTTTCGGCAACGCAAAGACA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>g2184</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>g2184.t1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>GAPDH; M5 glycolysis (expected flat)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.482484515353477</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>CCTGGTACGATAACGAGGCC</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>TAGGCCTGGCTGTTCATGTG</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>-6</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>CCTGGTACGATAACGAGGCCGGATACTCCGCCAAGTGCCTCGAGCTCATCCAGCACATGAACAGCCAGGCCTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>g6544</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>g6544.t1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Pyruvate kinase; M5 glycolysis (expected flat)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0.689648640096757</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>TAACACCCTCGCCAACATCC</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>CGTAGTCGGTGGTGATCTCG</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>164</v>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>-5</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>TAACACCCTCGCCAACATCCGCGCTGCCGCCGCTGAGCGCCCCGACCGCCAGGTCGCCGTGCTCCTCGACACCAAGGGCCCCGAGGTCCGCACGGGTTTCCTTGCCAACGGAGACCACGTTATGCTTCAGAAGGGTGCCCATGTCGAGATCACCACCGACTACG</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>g6030</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>g6030.t1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>SWEET-type sugar transporter; M5 glucose uptake</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0.00679755903379502</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>GTGCAACCGTTGGTTCTGTC</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>TTGCTGCCACAATGACAAGC</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>GTGCAACCGTTGGTTCTGTCTTGGGCGTTTTTTATTTACTTACAGCAATTAATCTTACAACGAGCAAGGAACAAGTCCGCAAAGTCGAGATATTTTTGCTTCCACAGCTTGTCATTGTGGCAGCAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>g4043</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>g4043.t1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>DnaJ chaperone; M6 heat-shock module</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>4.41420629285471e-89</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>AGCCAGCAGACATGGTCTTC</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>CGCGAATGTGGTGATTGTCC</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>AGCCAGCAGACATGGTCTTCAAACTCAAGGAAAAGCCCCATGAGGTCTTTACTCGCAAGGGCGATGATCTCTACACCACAATCGACGTCAGCCTTAAGGATGCCCTTATCGGCGGCAACGCTATCGTCAAAACTCTGGACAATCACCACATTCGCG</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>g6378</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>g6378.t1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ferric reductase; M6 iron module</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>3.55491083413054e-33</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>AGAACTACGTGCTCCAACCG</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>TCTTGGGTAGGTAGCGTCGA</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>same as cDNA (single exon: use no-RT control)</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>AGAACTACGTGCTCCAACCGGCCACCACCTGGGACTTCCAAACTGAACGCCCTGTTCGACGCTACCTACCCAAGA</t>
         </is>
       </c>
     </row>
@@ -3285,292 +3954,436 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>g1305</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>M3 Growth machinery: actin / myosin</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>Actin</t>
         </is>
       </c>
-      <c r="D34" s="12" t="n">
+      <c r="D34" s="10" t="n">
         <v>1716</v>
       </c>
-      <c r="E34" s="12" t="n">
+      <c r="E34" s="10" t="n">
         <v>-1.92</v>
       </c>
-      <c r="F34" s="12" t="n">
+      <c r="F34" s="10" t="n">
         <v>7.50108995036688e-20</v>
       </c>
-      <c r="G34" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H34" s="13" t="inlineStr"/>
-      <c r="I34" s="13" t="inlineStr"/>
-      <c r="J34" s="12" t="inlineStr"/>
-      <c r="K34" s="12" t="inlineStr"/>
-      <c r="L34" s="12" t="inlineStr"/>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>CCCATCTACGAGGGTTACGC</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>GTGGTGGTGAAGGAGTAGCC</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>119</v>
+      </c>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t>family-specific: 100% match at exactly the 4 actin loci, no other site; NOT g1305-specific</t>
+        </is>
+      </c>
+      <c r="L34" s="10" t="inlineStr">
+        <is>
+          <t>pan-actin: conserved in all 4 copies (g1305, g13337, g13659, g1757); measures total actin</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>g8048</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>M3 Growth machinery: actin / myosin</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>Myosin-6</t>
         </is>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D35" s="10" t="n">
         <v>436</v>
       </c>
-      <c r="E35" s="12" t="n">
+      <c r="E35" s="10" t="n">
         <v>-2.04</v>
       </c>
-      <c r="F35" s="12" t="n">
+      <c r="F35" s="10" t="n">
         <v>1.61906919291573e-10</v>
       </c>
-      <c r="G35" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H35" s="13" t="inlineStr"/>
-      <c r="I35" s="13" t="inlineStr"/>
-      <c r="J35" s="12" t="inlineStr"/>
-      <c r="K35" s="12" t="inlineStr"/>
-      <c r="L35" s="12" t="inlineStr"/>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>GTGCTTCAAGTTGTGGCAGG</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>AGGGCTCTTTCCAGTGCATC</t>
+        </is>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>164</v>
+      </c>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L35" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>g8072</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>M3 Growth machinery: actin / myosin</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Myosin-I heavy chain</t>
         </is>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D36" s="10" t="n">
         <v>256</v>
       </c>
-      <c r="E36" s="12" t="n">
+      <c r="E36" s="10" t="n">
         <v>-1.69</v>
       </c>
-      <c r="F36" s="12" t="n">
+      <c r="F36" s="10" t="n">
         <v>1.08697695779639e-07</v>
       </c>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H36" s="13" t="inlineStr"/>
-      <c r="I36" s="13" t="inlineStr"/>
-      <c r="J36" s="12" t="inlineStr"/>
-      <c r="K36" s="12" t="inlineStr"/>
-      <c r="L36" s="12" t="inlineStr"/>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>CTCAGCAAATCTTCGCGAGC</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>TGTCTTTGCGTTGCCGAAAG</t>
+        </is>
+      </c>
+      <c r="J36" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="K36" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L36" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>g2184</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>M5 Glucose uptake / glycolysis</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>Glyceraldehyde-3-phosphate dehydrogenase</t>
         </is>
       </c>
-      <c r="D37" s="12" t="n">
+      <c r="D37" s="10" t="n">
         <v>7223</v>
       </c>
-      <c r="E37" s="12" t="n">
+      <c r="E37" s="10" t="n">
         <v>-0.31</v>
       </c>
-      <c r="F37" s="12" t="n">
+      <c r="F37" s="10" t="n">
         <v>0.482484515353477</v>
       </c>
-      <c r="G37" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H37" s="13" t="inlineStr"/>
-      <c r="I37" s="13" t="inlineStr"/>
-      <c r="J37" s="12" t="inlineStr"/>
-      <c r="K37" s="12" t="inlineStr"/>
-      <c r="L37" s="12" t="inlineStr"/>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>CCTGGTACGATAACGAGGCC</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>TAGGCCTGGCTGTTCATGTG</t>
+        </is>
+      </c>
+      <c r="J37" s="10" t="n">
+        <v>73</v>
+      </c>
+      <c r="K37" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L37" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>g6544</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>M5 Glucose uptake / glycolysis</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>Pyruvate kinase</t>
         </is>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D38" s="10" t="n">
         <v>2873</v>
       </c>
-      <c r="E38" s="12" t="n">
+      <c r="E38" s="10" t="n">
         <v>-0.31</v>
       </c>
-      <c r="F38" s="12" t="n">
+      <c r="F38" s="10" t="n">
         <v>0.689648640096757</v>
       </c>
-      <c r="G38" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H38" s="13" t="inlineStr"/>
-      <c r="I38" s="13" t="inlineStr"/>
-      <c r="J38" s="12" t="inlineStr"/>
-      <c r="K38" s="12" t="inlineStr"/>
-      <c r="L38" s="12" t="inlineStr"/>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>TAACACCCTCGCCAACATCC</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>CGTAGTCGGTGGTGATCTCG</t>
+        </is>
+      </c>
+      <c r="J38" s="10" t="n">
+        <v>164</v>
+      </c>
+      <c r="K38" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L38" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>g6030</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>M5 Glucose uptake / glycolysis</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Bidirectional sugar transporter SWEET6</t>
         </is>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D39" s="10" t="n">
         <v>187</v>
       </c>
-      <c r="E39" s="12" t="n">
+      <c r="E39" s="10" t="n">
         <v>-1.19</v>
       </c>
-      <c r="F39" s="12" t="n">
+      <c r="F39" s="10" t="n">
         <v>0.00679755903379502</v>
       </c>
-      <c r="G39" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H39" s="13" t="inlineStr"/>
-      <c r="I39" s="13" t="inlineStr"/>
-      <c r="J39" s="12" t="inlineStr"/>
-      <c r="K39" s="12" t="inlineStr"/>
-      <c r="L39" s="12" t="inlineStr"/>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>GTGCAACCGTTGGTTCTGTC</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>TTGCTGCCACAATGACAAGC</t>
+        </is>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>126</v>
+      </c>
+      <c r="K39" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L39" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>g4043</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>M6 Largest unexplained responses</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>DnaJ homolog subfamily B member 5</t>
         </is>
       </c>
-      <c r="D40" s="12" t="n">
+      <c r="D40" s="10" t="n">
         <v>2669</v>
       </c>
-      <c r="E40" s="12" t="n">
+      <c r="E40" s="10" t="n">
         <v>4.65</v>
       </c>
-      <c r="F40" s="12" t="n">
+      <c r="F40" s="10" t="n">
         <v>4.41420629285471e-89</v>
       </c>
-      <c r="G40" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H40" s="13" t="inlineStr"/>
-      <c r="I40" s="13" t="inlineStr"/>
-      <c r="J40" s="12" t="inlineStr"/>
-      <c r="K40" s="12" t="inlineStr"/>
-      <c r="L40" s="12" t="inlineStr"/>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>AGCCAGCAGACATGGTCTTC</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>CGCGAATGTGGTGATTGTCC</t>
+        </is>
+      </c>
+      <c r="J40" s="10" t="n">
+        <v>156</v>
+      </c>
+      <c r="K40" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L40" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>g6378</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>M6 Largest unexplained responses</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>Ferric reduction oxidase 7, chloroplastic</t>
         </is>
       </c>
-      <c r="D41" s="12" t="n">
+      <c r="D41" s="10" t="n">
         <v>325</v>
       </c>
-      <c r="E41" s="12" t="n">
+      <c r="E41" s="10" t="n">
         <v>3.48</v>
       </c>
-      <c r="F41" s="12" t="n">
+      <c r="F41" s="10" t="n">
         <v>3.55491083413054e-33</v>
       </c>
-      <c r="G41" s="12" t="inlineStr">
-        <is>
-          <t>PROPOSED: primers not yet designed</t>
-        </is>
-      </c>
-      <c r="H41" s="13" t="inlineStr"/>
-      <c r="I41" s="13" t="inlineStr"/>
-      <c r="J41" s="12" t="inlineStr"/>
-      <c r="K41" s="12" t="inlineStr"/>
-      <c r="L41" s="12" t="inlineStr"/>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>NEW (this update)</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>AGAACTACGTGCTCCAACCG</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>TCTTGGGTAGGTAGCGTCGA</t>
+        </is>
+      </c>
+      <c r="J41" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="K41" s="10" t="inlineStr">
+        <is>
+          <t>unique: 1 genome site per primer, no extra predicted amplicon</t>
+        </is>
+      </c>
+      <c r="L41" s="10" t="inlineStr">
+        <is>
+          <t>no junction spanned (needs no-RT control)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3583,7 +4396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3646,7 +4459,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>g6055, g845 and g1664 have repeat-built coding sequence: most candidate primers match several near-identical genomic sites. In 200 candidates, g845 had no pair passing, g1664 had one and g6055 three. See the status column; a NOT-unique primer must not be used for quantification without amplicon sequencing and a melt curve, or a design in a unique 3' UTR (needs RNA-seq-based UTR mapping).</t>
+          <t>g6055, g845 and g1664 have repeat-built coding sequence: most candidate primers match several near-identical genomic sites. In 200 candidates, g845 had no pair passing, g1664 had one and g6055 three. Actin (g1305) has three near-identical copies (g13337, g13659, g1757; 99.3-99.6% identical, all down in HS6), so the actin pair is a deliberate pan-actin design that matches all four copies at 100% and measures TOTAL actin; it cannot isolate g1305. See the status column; a NOT-unique primer must not be used for quantification without amplicon sequencing and a melt curve, or a design in a unique 3' UTR (needs RNA-seq-based UTR mapping).</t>
         </is>
       </c>
     </row>
@@ -3665,10 +4478,34 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>Sequence differences (eight genes added 2026-10-08)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>SKKU no-filter comparison: zero HS6-vs-#4 sequence differences in the gene body, CDS or introns of g1305, g8048, g8072, g2184, g6544, g6030, g4043 and g6378, so the primers cannot be affected by genotype-specific SNPs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sequence differences (eight genes added 2026-10-08)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SKKU no-filter comparison: zero HS6-vs-#4 sequence differences in the gene body, CDS or introns of g1305, g8048, g8072, g2184, g6544, g6030, g4043 and g6378, so the primers cannot be affected by genotype-specific SNPs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Existing panel check</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>The older 27-pair panel was re-checked today with the same strict genome test: 26 clean, 1 modest (g3889). Tm under standard conditions 59.6-60.1 C, products 72-199 bp.</t>
         </is>

</xml_diff>